<commit_message>
Riparazione province e Bassano
</commit_message>
<xml_diff>
--- a/web/Pipistrelli 2025.xlsx
+++ b/web/Pipistrelli 2025.xlsx
@@ -7989,9 +7989,17 @@
           <t>Carrè</t>
         </is>
       </c>
-      <c r="G135" t="inlineStr"/>
-      <c r="H135" t="inlineStr"/>
-      <c r="I135" t="inlineStr"/>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>VI</t>
+        </is>
+      </c>
+      <c r="H135" t="n">
+        <v>45.51732904101443</v>
+      </c>
+      <c r="I135" t="n">
+        <v>11.57734365722946</v>
+      </c>
       <c r="J135" t="inlineStr">
         <is>
           <t>cucciolo</t>
@@ -8373,9 +8381,17 @@
           <t>Santorso</t>
         </is>
       </c>
-      <c r="G142" t="inlineStr"/>
-      <c r="H142" t="inlineStr"/>
-      <c r="I142" t="inlineStr"/>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>VI</t>
+        </is>
+      </c>
+      <c r="H142" t="n">
+        <v>45.51722487863642</v>
+      </c>
+      <c r="I142" t="n">
+        <v>11.56642781741572</v>
+      </c>
       <c r="J142" t="inlineStr">
         <is>
           <t>cucciolo</t>
@@ -12997,9 +13013,17 @@
           <t>Sossano</t>
         </is>
       </c>
-      <c r="G225" t="inlineStr"/>
-      <c r="H225" t="inlineStr"/>
-      <c r="I225" t="inlineStr"/>
+      <c r="G225" t="inlineStr">
+        <is>
+          <t>VI</t>
+        </is>
+      </c>
+      <c r="H225" t="n">
+        <v>45.58468152873789</v>
+      </c>
+      <c r="I225" t="n">
+        <v>11.54923228109381</v>
+      </c>
       <c r="J225" t="inlineStr">
         <is>
           <t>adulto</t>

</xml_diff>